<commit_message>
funcional antes de opt
</commit_message>
<xml_diff>
--- a/output/xlsx/matriz_entrada_codificacion.xlsx
+++ b/output/xlsx/matriz_entrada_codificacion.xlsx
@@ -430,7 +430,7 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,7 +612,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar la reserva asociándola al estudiante autenticado, incluyendo el ejemplar seleccionado y la fecha y hora de la operación.</t>
+          <t>El sistema deberá registrar la reserva asociándola al estudiante autenticado, el ejemplar seleccionado y la fecha y hora de la operación.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Impedir reserva de ejemplar con reserva activa</t>
+          <t>Impedir reservas duplicadas activas</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DIS-002</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CORREGIR</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DIS-002</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -783,17 +783,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CORREGIR</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la disponibilidad inmediatamente después de confirmar una reserva.</t>
+          <t>El sistema deberá actualizar la disponibilidad del ejemplar inmediatamente después de confirmar una reserva.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Un ejemplar solo puede tener una reserva activa simultáneamente</t>
+          <t>Reservar un ejemplar disponible del catálogo de la biblioteca</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá un ejemplar solo puede tener una reserva activa simultáneamente.</t>
+          <t>El sistema deberá reservar un ejemplar disponible del catálogo de la biblioteca.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -971,12 +971,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
+          <t>Un ejemplar solo puede tener una reserva activa simultáneamente</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
+          <t>El sistema deberá un ejemplar solo puede tener una reserva activa simultáneamente.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>La operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación</t>
+          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación.</t>
+          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la información del préstamo después de la devolución.</t>
+          <t>El sistema deberá actualizar la información del préstamo después de registrar la devolución.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir continuar con el proceso cuando los datos sean correctos.</t>
+          <t>El sistema deberá permitir continuar con el proceso cuando los datos de la devolución sean correctos.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">

</xml_diff>

<commit_message>
cambio a modelo nuevo por deprecacion de glm5.2
</commit_message>
<xml_diff>
--- a/output/xlsx/matriz_entrada_codificacion.xlsx
+++ b/output/xlsx/matriz_entrada_codificacion.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad Diseño" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trazabilidad Diseño'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trazabilidad Diseño'!$A$1:$J$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -429,8 +429,8 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="56" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,7 +503,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mostrar ejemplares disponibles para reserva</t>
+          <t>Consulta de ejemplares disponibles</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CONFORME CON MEJORAS</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mostrar información del ejemplar antes de confirmar</t>
+          <t>Visualización de detalles del ejemplar</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CONFORME CON MEJORAS</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J3" s="1" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Registrar reserva del ejemplar</t>
+          <t>Registro de reserva</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CONFORME CON MEJORAS</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cambiar estado del ejemplar a reservado</t>
+          <t>Actualización de estado del ejemplar</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CONFORME CON MEJORAS</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Impedir reservas duplicadas activas</t>
+          <t>Bloqueo de reserva duplicada</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -721,27 +721,27 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mostrar confirmación de reserva</t>
+          <t>Confirmación de reserva</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -773,27 +773,27 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Informar fecha límite de recogida</t>
+          <t>Información de fecha límite de recogida</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -825,27 +825,27 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J8" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -867,37 +867,37 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Actualización inmediata de disponibilidad</t>
+          <t>Inmediatez en la actualización de disponibilidad</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la disponibilidad del ejemplar inmediatamente después de confirmar una reserva.</t>
+          <t>El sistema deberá actualizar la disponibilidad inmediatamente después de confirmar una reserva.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -919,37 +919,37 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Reservar un ejemplar disponible del catálogo de la biblioteca</t>
+          <t>Un ejemplar solo puede tener una reserva activa simultáneamente</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá reservar un ejemplar disponible del catálogo de la biblioteca.</t>
+          <t>El sistema deberá un ejemplar solo puede tener una reserva activa simultáneamente.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -971,37 +971,37 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Un ejemplar solo puede tener una reserva activa simultáneamente</t>
+          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá un ejemplar solo puede tener una reserva activa simultáneamente.</t>
+          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1023,37 +1023,37 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
+          <t>El sistema debe impedir la reserva cuando el ejemplar no se encuentre disponible</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
+          <t>El sistema deberá el sistema debe impedir la reserva cuando el ejemplar no se encuentre disponible.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-001</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONFORME</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1085,27 +1085,27 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01, ED-02</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1137,27 +1137,27 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1189,27 +1189,27 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02, ED-04</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1241,27 +1241,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1283,37 +1283,37 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Continuar proceso con datos correctos</t>
+          <t>Permitir continuar proceso con datos correctos</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir continuar con el proceso cuando los datos de la devolución sean correctos.</t>
+          <t>El sistema deberá permitir continuar con el proceso cuando los datos sean correctos.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1345,27 +1345,27 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>DIS-002</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Pendiente de relación</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
         </is>
       </c>
     </row>
@@ -1397,27 +1397,27 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-03</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1449,27 +1449,27 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DIS-002</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-03</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>No evaluado</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CORREGIR</t>
         </is>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1501,32 +1501,448 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>DIS-002</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Pendiente de relación</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="inlineStr">
+        <is>
+          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RF-021</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Consultar historial de préstamos del estudiante</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá mostrar únicamente los préstamos asociados al estudiante autenticado que realiza la consulta.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ED-01, ED-02, ED-03</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Cubierto en Diseño</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con evidencia suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RF-022</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ordenar historial de préstamos por fecha</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá presentar la lista de préstamos ordenada por fecha, del más reciente al más antiguo.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ED-01</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Cubierto en Diseño</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con evidencia suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RF-023</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mostrar detalles del préstamo en el historial</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá mostrar para cada préstamo el título del libro, la fecha de préstamo, la fecha de devolución esperada y el estado actual.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ED-01</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Cubierto en Diseño</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con evidencia suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>RF-024</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Filtrar préstamos por estado</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá permitir filtrar los préstamos del historial por estado.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ED-01</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Cubierto en Diseño</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con evidencia suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RF-025</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mostrar mensaje de historial vacío</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá mostrar un mensaje cuando el estudiante no tenga préstamos registrados.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ED-02</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Cubierto en Diseño</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con evidencia suficiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RF-026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Impedir consulta de historial ajeno</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá impedir que un estudiante consulte el historial de otro estudiante.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>No evaluado</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Pendiente de relación</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="inlineStr">
+        <is>
+          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RF-027</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>La información mostrada debe reflejar el estado actual de cada préstamo</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá la información mostrada debe reflejar el estado actual de cada préstamo.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J21" s="1" t="inlineStr">
-        <is>
-          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Pendiente de relación</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RF-028</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No se permite la modificación de los registros desde esta consulta</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá no se permite la modificación de los registros desde esta consulta.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Pendiente de relación</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:J29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
arreglo de modelos cod y pru
</commit_message>
<xml_diff>
--- a/output/xlsx/matriz_entrada_codificacion.xlsx
+++ b/output/xlsx/matriz_entrada_codificacion.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad Diseño" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trazabilidad Diseño'!$A$1:$J$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trazabilidad Diseño'!$A$1:$J$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -503,7 +503,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Consulta de ejemplares disponibles</t>
+          <t>Mostrar ejemplares disponibles para reserva</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -513,27 +513,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ED-01, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Visualización de detalles del ejemplar</t>
+          <t>Mostrar detalles del ejemplar antes de confirmar reserva</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -565,27 +565,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -607,37 +607,37 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Registro de reserva</t>
+          <t>Registrar reserva asociada al estudiante autenticado</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar la reserva asociándola al estudiante autenticado, el ejemplar seleccionado y la fecha y hora de la operación.</t>
+          <t>El sistema deberá registrar la reserva asociándola al estudiante autenticado.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ED-02, ED-04</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Actualización de estado del ejemplar</t>
+          <t>Cambiar estado del ejemplar a reservado</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -669,27 +669,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bloqueo de reserva duplicada</t>
+          <t>Impedir reserva de ejemplar con reserva activa</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -721,27 +721,27 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Confirmación de reserva</t>
+          <t>Mostrar confirmación de reserva registrada</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -773,27 +773,27 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Información de fecha límite de recogida</t>
+          <t>Informar fecha límite para recoger ejemplar</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -825,27 +825,27 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J8" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -867,37 +867,37 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Inmediatez en la actualización de disponibilidad</t>
+          <t>Reservar un ejemplar disponible del catálogo de la biblioteca</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la disponibilidad inmediatamente después de confirmar una reserva.</t>
+          <t>El sistema deberá reservar un ejemplar disponible del catálogo de la biblioteca.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -929,27 +929,27 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -971,37 +971,37 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
+          <t>La disponibilidad debe actualizarse inmediatamente después de confirmar una reserva</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
+          <t>El sistema deberá la disponibilidad debe actualizarse inmediatamente después de que el estudiante confirme una reserva.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ED-02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
@@ -1023,44 +1023,44 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>El sistema debe impedir la reserva cuando el ejemplar no se encuentre disponible</t>
+          <t>La reserva debe quedar asociada al estudiante que realizó la operación</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá el sistema debe impedir la reserva cuando el ejemplar no se encuentre disponible.</t>
+          <t>El sistema deberá la reserva debe quedar asociada al estudiante que realizó la operación.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>DIS-001</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>No evaluado</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CONFORME</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
+          <t>HU-001 – HU-001 - Reservar libro disponible</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Registrar devolución de libro</t>
+          <t>La operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir registrar la devolución de un libro prestado.</t>
+          <t>El sistema deberá la operación de reserva debe utilizar la disponibilidad actual del ejemplar. Se debe registrar el estudiante que realizó la reserva, el ejemplar seleccionado y la fecha y hora de la operación.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>ED-01, ED-02</t>
+          <t>ED-02, ED-03, ED-04</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>Requiere revisión</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
         </is>
       </c>
     </row>
@@ -1127,12 +1127,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Verificar préstamo relacionado</t>
+          <t>Registrar devolución de libro</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá verificar que exista un préstamo relacionado con el libro al registrar su devolución.</t>
+          <t>El sistema deberá permitir registrar la devolución de un libro.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>ED-02, ED-03</t>
+          <t>ED-01, ED-02, ED-04</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1179,12 +1179,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Actualizar información del préstamo</t>
+          <t>Verificar existencia de préstamo</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá actualizar la información del préstamo después de registrar la devolución.</t>
+          <t>El sistema deberá verificar que exista un préstamo relacionado con el libro.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ED-02, ED-04</t>
+          <t>ED-02, ED-03</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Mostrar mensaje de confirmación de devolución</t>
+          <t>Actualizar información del préstamo</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar un mensaje cuando la devolución haya sido registrada.</t>
+          <t>El sistema deberá actualizar la información del préstamo después de la devolución.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>ED-02, ED-04</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Permitir continuar proceso con datos correctos</t>
+          <t>Mostrar mensaje de devolución registrada</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir continuar con el proceso cuando los datos sean correctos.</t>
+          <t>El sistema deberá mostrar un mensaje cuando la devolución haya sido registrada.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>ED-01, ED-02</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Registrar mascota</t>
+          <t>Continuar proceso con datos correctos</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar mascota.</t>
+          <t>El sistema deberá permitir continuar con el proceso cuando los datos sean correctos.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1387,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>El libro debe existir en el sistema</t>
+          <t>Registrar mascota</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá el libro debe existir en el sistema.</t>
+          <t>El sistema deberá registrar mascota.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>La devolución debe corresponder a un préstamo registrado</t>
+          <t>El libro debe existir en el sistema</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la devolución debe corresponder a un préstamo registrado.</t>
+          <t>El sistema deberá el libro debe existir en el sistema.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación</t>
+          <t>La devolución debe corresponder a un préstamo registrado</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación.</t>
+          <t>El sistema deberá la devolución debe corresponder a un préstamo registrado.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1506,12 +1506,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-03</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1521,14 +1521,14 @@
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HU-003 – HU-003 Consultar historial</t>
+          <t>HU-002 – HU-002 - Registrar préstamo de libro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Consultar historial de préstamos del estudiante</t>
+          <t>Todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar únicamente los préstamos asociados al estudiante autenticado que realiza la consulta.</t>
+          <t>El sistema deberá todavía no se ha definido qué información específica debe actualizarse al registrar la devolución, cómo se manejarán las devoluciones realizadas fuera de plazo ni qué información deberá conservarse como evidencia de la operación.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ED-01, ED-02, ED-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>Requiere revisión</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
         </is>
       </c>
     </row>
@@ -1595,12 +1595,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ordenar historial de préstamos por fecha</t>
+          <t>Consultar historial de préstamos</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá presentar la lista de préstamos ordenada por fecha, del más reciente al más antiguo.</t>
+          <t>El sistema deberá consultar el historial de los préstamos que el estudiante autenticado ha realizado en la biblioteca.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ED-01</t>
+          <t>ED-01, ED-02, ED-03</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Mostrar detalles del préstamo en el historial</t>
+          <t>Mostrar préstamos del estudiante autenticado</t>
         </is>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar para cada préstamo el título del libro, la fecha de préstamo, la fecha de devolución esperada y el estado actual.</t>
+          <t>El sistema deberá mostrar únicamente los préstamos asociados al estudiante autenticado.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>Requiere revisión</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
         </is>
       </c>
     </row>
@@ -1699,12 +1699,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Filtrar préstamos por estado</t>
+          <t>Ordenar préstamos por fecha descendente</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir filtrar los préstamos del historial por estado.</t>
+          <t>El sistema deberá presentar la lista de préstamos ordenada por fecha, del más reciente al más antiguo.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>Requiere revisión</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mostrar mensaje de historial vacío</t>
+          <t>Mostrar detalles de cada préstamo</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá mostrar un mensaje cuando el estudiante no tenga préstamos registrados.</t>
+          <t>El sistema deberá mostrar para cada préstamo el título del libro, la fecha de préstamo, la fecha de devolución esperada y el estado actual (activo, devuelto, vencido).</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1766,12 +1766,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ED-02</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Cubierto en Diseño</t>
+          <t>Requiere revisión</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>Relación identificada con evidencia suficiente.</t>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
         </is>
       </c>
     </row>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Impedir consulta de historial ajeno</t>
+          <t>Filtrar préstamos por estado</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá impedir que un estudiante consulte el historial de otro estudiante.</t>
+          <t>El sistema deberá permitir filtrar los préstamos por estado.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1818,12 +1818,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-01</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>La información mostrada debe reflejar el estado actual de cada préstamo</t>
+          <t>Mostrar mensaje sin préstamos</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>El sistema deberá la información mostrada debe reflejar el estado actual de cada préstamo.</t>
+          <t>El sistema deberá mostrar un mensaje cuando el estudiante no tenga préstamos registrados.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ED-02</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Pendiente de relación</t>
+          <t>Cubierto en Diseño</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+          <t>Relación identificada con evidencia suficiente.</t>
         </is>
       </c>
     </row>
@@ -1907,42 +1907,146 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>Impedir que un estudiante consulte el historial de otro estudiante</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá impedir que un estudiante consulte el historial de otro estudiante.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DIS-003</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Requiere revisión</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CORREGIR</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>Relación identificada con confianza insuficiente para confirmarla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RF-029</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>La información mostrada debe reflejar el estado actual de cada préstamo</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>El sistema deberá la información mostrada debe reflejar el estado actual de cada préstamo.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>No evaluado</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr">
+        <is>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HU-003 – HU-003 Consultar historial</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RF-030</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>No se permite la modificación de los registros desde esta consulta</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>El sistema deberá no se permite la modificación de los registros desde esta consulta.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>DIS-003</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Pendiente de relación</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>CORREGIR</t>
-        </is>
-      </c>
-      <c r="J29" s="1" t="inlineStr">
-        <is>
-          <t>No se identificó evidencia suficiente para asociarlo a un elemento de diseño.</t>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No evaluado</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr">
+        <is>
+          <t>No se evaluó este requisito en ningún Issue de Diseño.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J29"/>
+  <autoFilter ref="A1:J31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>